<commit_message>
Update accident data and map simulation
Added a new entry to accident_data.csv and updated accident_report.xlsx. Updated road_accident_map_simulation.html with new map element IDs and revised map data coordinates and elevations for improved simulation accuracy.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,7 +651,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Head-on collision</t>
+          <t>Vehicle-pedestrian collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2.64 seconds</t>
+          <t>1.68 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Drunk Driving</t>
+          <t>Mechanical Failure</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,28 +675,24 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1297</v>
+        <v>1249</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>56.5</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Car 2</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>1493</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>-73.0</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
+          <t>81.3</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Pedestrian</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>77</v>
+      </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
           <t>wet</t>
@@ -713,16 +709,16 @@
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>180</v>
+        <v>15</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2.64</t>
+          <t>1.68</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>2547317.09</t>
+          <t>179950.02</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
@@ -740,21 +736,21 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Install median barriers
-- Public awareness campaigns on drinking and driving
-- Solar-powered lighting solutions
-- Weather-based speed limit adjustments
-- Stricter DUI checkpoints</t>
+          <t>- Solar-powered lighting solutions
+- Improve maintenance education
+- Improve drainage systems
+- Install pedestrian crossings
+- Mandatory vehicle inspections</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Driver state (Under influence) affected reaction time (Impaired decision making due to alcohol or substances.); Road geometry (straight) with wet surface influenced braking distance; Limited lighting stretched driver perception; Primary cause flagged: Drunk Driving; Interventions tested: speed checkpoint, driver safety campaign, improved street lighting, road surface treatment.</t>
+          <t>Driver state (Under influence) affected reaction time (Impaired decision making due to alcohol or substances.); Road geometry (straight) with wet surface influenced braking distance; Limited lighting stretched driver perception; Primary cause flagged: Mechanical Failure; Interventions tested: speed checkpoint, driver safety campaign, improved street lighting, road surface treatment.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>85.7% of historical accidents in Main Highway share severe severity.</t>
+          <t>87.2% of historical accidents in Main Highway share severe severity.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -769,22 +765,22 @@
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>2547317.09</t>
+          <t>179950.02</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>2090035.85</t>
+          <t>134962.52</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>17.95%</t>
+          <t>25.00%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update accident data and simulation map
Added new accident records to accident_data.csv and updated accident_report.xlsx. Modified road_accident_map_simulation.html to update map element IDs and deckData coordinates, reflecting new simulation data. No changes to simulation logic in road_accident_simulation.py are shown.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -651,7 +651,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Vehicle-pedestrian collision</t>
+          <t>Head-on collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1.68 seconds</t>
+          <t>2.86 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -675,24 +675,28 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1249</v>
+        <v>1218</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>81.3</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Pedestrian</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>77</v>
-      </c>
+          <t>62.5</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Car 2</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1241</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>-57.1</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
           <t>wet</t>
@@ -709,16 +713,16 @@
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>15</v>
+        <v>180</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>179950.02</t>
+          <t>2082317.08</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
@@ -736,21 +740,21 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Solar-powered lighting solutions
-- Improve maintenance education
-- Improve drainage systems
-- Install pedestrian crossings
+          <t>- Weather-based speed limit adjustments
+- Upgrade to LED lighting systems
+- Create emergency roadside assistance programs
+- One-way traffic in narrow roads
 - Mandatory vehicle inspections</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Driver state (Under influence) affected reaction time (Impaired decision making due to alcohol or substances.); Road geometry (straight) with wet surface influenced braking distance; Limited lighting stretched driver perception; Primary cause flagged: Mechanical Failure; Interventions tested: speed checkpoint, driver safety campaign, improved street lighting, road surface treatment.</t>
+          <t>Mechanical failure in vehicle systems interacts with human response capabilities and road conditions, creating unexpected hazards in systems theory.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>87.2% of historical accidents in Main Highway share severe severity.</t>
+          <t>88.1% of historical accidents in Main Highway share severe severity.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -765,22 +769,22 @@
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>179950.02</t>
+          <t>2082317.08</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>134962.52</t>
+          <t>1685958.92</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>19.03%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Refactor HTML to use external CSS for map simulation
Moved all CSS styles from road_accident_map_simulation.html to a new external stylesheet road_accident_map_simulation.css for better maintainability. Updated HTML to reference the new CSS file and cleaned up redundant inline styles. Also added new accident and vehicle data to accident_data.csv and cache, and updated accident_report.xlsx and Python files for simulation output.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,7 +651,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Head-on collision</t>
+          <t>Rear-end collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2.86 seconds</t>
+          <t>10.01 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Mechanical Failure</t>
+          <t>Poor Visibility</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1218</v>
+        <v>1275</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>62.5</t>
+          <t>94.4</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -688,11 +688,11 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1241</v>
+        <v>1412</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>-57.1</t>
+          <t>86.3</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
@@ -713,25 +713,25 @@
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>10.01</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>2082317.08</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>10</v>
+        <v>2.1</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -740,21 +740,21 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Weather-based speed limit adjustments
-- Upgrade to LED lighting systems
-- Create emergency roadside assistance programs
-- One-way traffic in narrow roads
-- Mandatory vehicle inspections</t>
+          <t>- Solar-powered lighting solutions
+- Improve weather-responsive lighting systems
+- Increase following distance education
+- Weather-based speed limit adjustments
+- Upgrade street lighting</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Mechanical failure in vehicle systems interacts with human response capabilities and road conditions, creating unexpected hazards in systems theory.</t>
+          <t>Poor visibility limits human perception, interacting with vehicle lighting and road markings in systems theory to compromise safety margins.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>88.1% of historical accidents in Main Highway share severe severity.</t>
+          <t>0.0% of historical accidents in Main Highway share none severity.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -764,42 +764,42 @@
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>2082317.08</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>1685958.92</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>19.03%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
+          <t>1.97 (Baseline 2.10, Intervention 0.13)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new accident data and enhance map UI
Added a new record for drunk driving in accident_data.csv and updated accident_report.xlsx. Refactored road_accident_map_simulation.css to move control panel and legend styles from inline to stylesheet, and added new marker and collision effect styles in road_accident_map_simulation.html for improved map visualization and UI consistency.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,7 +651,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Rear-end collision</t>
+          <t>Head-on collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>10.01 seconds</t>
+          <t>2.26 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Poor Visibility</t>
+          <t>Drunk Driving</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1275</v>
+        <v>1356</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>94.4</t>
+          <t>82.1</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -688,11 +688,11 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1412</v>
+        <v>1313</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>86.3</t>
+          <t>-68.7</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
@@ -713,25 +713,25 @@
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>10.01</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2850409.54</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>2.1</v>
+        <v>10</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -741,20 +741,20 @@
       <c r="V4" s="3" t="inlineStr">
         <is>
           <t>- Solar-powered lighting solutions
-- Improve weather-responsive lighting systems
-- Increase following distance education
 - Weather-based speed limit adjustments
-- Upgrade street lighting</t>
+- Stricter DUI checkpoints
+- Improve lane markings
+- Public awareness campaigns on drinking and driving</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Poor visibility limits human perception, interacting with vehicle lighting and road markings in systems theory to compromise safety margins.</t>
+          <t>Drunk driving impairs human judgment and reaction time, interacting with vehicle control systems and road geometry to create hazardous situations in systems theory.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>0.0% of historical accidents in Main Highway share none severity.</t>
+          <t>88.1% of historical accidents in Main Highway share severe severity.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -764,42 +764,42 @@
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2850409.54</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2300233.04</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>19.30%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>1.97 (Baseline 2.10, Intervention 0.13)</t>
+          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>10.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add road accident simulation and analysis modules
Introduces core Python modules for road accident simulation, analysis, reporting, and machine learning-based severity prediction. Adds Streamlit dashboard (app.py), simulation logic (main.py, simulation.py), data models (models.py), constants, utilities, and reporting/visualization tools. Updates accident_data.csv and accident_report.xlsx with new records. Renames road_accident_simulation.py to road_accident_simulation_original.py.backup. Includes requirements.txt for dependencies.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,22 +651,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Head-on collision</t>
+          <t>Rear-end collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Main Highway, Labo, Camarines Norte</t>
+          <t>Bayabas, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2.26 seconds</t>
+          <t>10.01 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Drunk Driving</t>
+          <t>Overspeeding</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1356</v>
+        <v>1447</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>82.1</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -688,50 +688,50 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1313</v>
+        <v>1492</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>-68.7</t>
+          <t>105.9</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>wet</t>
+          <t>dry</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>poor</t>
+          <t>good</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Rainy</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>10.01</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>2850409.54</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>10</v>
+        <v>0.95</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -740,66 +740,66 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Solar-powered lighting solutions
-- Weather-based speed limit adjustments
-- Stricter DUI checkpoints
-- Improve lane markings
-- Public awareness campaigns on drinking and driving</t>
+          <t>- Regular road maintenance
+- Implement speed cameras
+- Maintain current lighting standards
+- Add speed bumps in high-risk areas
+- Install rear-end collision warning systems</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Drunk driving impairs human judgment and reaction time, interacting with vehicle control systems and road geometry to create hazardous situations in systems theory.</t>
+          <t>Overspeeding amplifies the impact of poor road conditions and reduces reaction time, leading to severe collisions in systems theory where human factors interact with vehicle dynamics and environmental constraints.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>88.1% of historical accidents in Main Highway share severe severity.</t>
+          <t>Historical validation unavailable.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Speed Checkpoint, Driver Safety Campaign, Improved Street Lighting, Road Surface Treatment</t>
+          <t>Road Surface Treatment, Improved Street Lighting, Speed Checkpoint</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>2850409.54</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>2300233.04</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>19.30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
+          <t>0.00 (Baseline 0.95, Intervention 0.95)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine Code, and Add New Barangays
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,22 +651,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Side-impact (T-bone) collision</t>
+          <t>Rear-end collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Main Highway, Labo, Camarines Norte</t>
+          <t>Bayabas, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2.24 seconds</t>
+          <t>10.01 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Drunk Driving</t>
+          <t>Overspeeding</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1274</v>
+        <v>1308</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -688,46 +688,50 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1305</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr"/>
+        <v>1428</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>71.3</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>wet</t>
+          <t>dry</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>poor</t>
+          <t>good</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Rainy</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2.24</t>
+          <t>10.01</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>1672226.88</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>10</v>
+        <v>0.95</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -736,66 +740,66 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Improve drainage systems
-- Stricter DUI checkpoints
-- Public awareness campaigns on drinking and driving
-- Enhanced crosswalk protections
-- Upgrade to LED lighting systems</t>
+          <t>- Add speed bumps in high-risk areas
+- Regular road maintenance
+- Increase following distance education
+- Increase speed limit enforcement
+- Maintain current lighting standards</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Drunk driving impairs human judgment and reaction time, interacting with vehicle control systems and road geometry to create hazardous situations in systems theory.</t>
+          <t>Overspeeding amplifies the impact of poor road conditions and reduces reaction time, leading to severe collisions in systems theory where human factors interact with vehicle dynamics and environmental constraints.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>88.9% of historical accidents in Main Highway share severe severity.</t>
+          <t>Historical validation unavailable.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Speed Checkpoint, Driver Safety Campaign, Improved Street Lighting, Road Surface Treatment</t>
+          <t>Road Surface Treatment, Improved Street Lighting, Speed Checkpoint</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>1672226.88</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>1254047.54</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>25.01%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
+          <t>0.00 (Baseline 0.95, Intervention 0.95)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add VSCode Python test settings and update GIS data
Added .vscode/settings.json to configure Python unittest discovery. Updated GIS/labo_roads.geojson with new and modified road features, including changes to barangay assignments and geometry. Other files show updates to code, data, and tests, but the main change is the addition of editor settings and GIS data refinement.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -651,22 +651,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Rear-end collision</t>
+          <t>Side-impact (T-bone) collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Bayabas, Labo, Camarines Norte</t>
+          <t>Malaya, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>10.01 seconds</t>
+          <t>2.53 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Overspeeding</t>
+          <t>Drunk Driving</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1308</v>
+        <v>1375</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>65.3</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -688,50 +688,46 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1428</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>71.3</t>
-        </is>
-      </c>
+        <v>1351</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>dry</t>
+          <t>wet</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>poor</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Rainy</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>10.01</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1538462.92</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>0.95</v>
+        <v>10</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -740,66 +736,66 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Add speed bumps in high-risk areas
-- Regular road maintenance
-- Increase following distance education
-- Increase speed limit enforcement
-- Maintain current lighting standards</t>
+          <t>- Improve drainage systems
+- Stricter DUI checkpoints
+- Install turning signal cameras
+- Install additional street lights
+- Public awareness campaigns on drinking and driving</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Overspeeding amplifies the impact of poor road conditions and reduces reaction time, leading to severe collisions in systems theory where human factors interact with vehicle dynamics and environmental constraints.</t>
+          <t>Drunk driving impairs human judgment and reaction time, interacting with vehicle control systems and road geometry to create hazardous situations in systems theory.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Historical validation unavailable.</t>
+          <t>No recorded accidents in Malaya for validation.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Road Surface Treatment, Improved Street Lighting, Speed Checkpoint</t>
+          <t>Improved Street Lighting, Road Surface Treatment, Speed Checkpoint</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1538462.92</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1153704.16</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25.01%</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>0.00 (Baseline 0.95, Intervention 0.95)</t>
+          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>10.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add results analysis notebook and update accident data
Added results_analysis.ipynb for simulation and accident data analysis. Updated accident_data.csv and accident_report.xlsx with new entries. Removed obsolete test files test_fps_html.py and test_map_call.py.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -462,7 +462,7 @@
     <col width="30" customWidth="1" min="22" max="22"/>
     <col width="30" customWidth="1" min="23" max="23"/>
     <col width="30" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="23" customWidth="1" min="27" max="27"/>
     <col width="27" customWidth="1" min="28" max="28"/>
@@ -651,22 +651,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Side-impact (T-bone) collision</t>
+          <t>Rear-end collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Santa Cruz, Labo, Camarines Norte</t>
+          <t>Main Highway, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2.75 seconds</t>
+          <t>10.01 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Fatigue</t>
+          <t>Drunk Driving</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1415</v>
+        <v>1362</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -688,14 +688,18 @@
         </is>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1479</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr"/>
+        <v>1343</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>93.6</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>wet</t>
+          <t>dry</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -705,29 +709,29 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Foggy</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>10.01</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>1155982.60</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -736,16 +740,16 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Campaigns on driver fatigue awareness
-- Maintain current lighting standards
-- Enhanced crosswalk protections
-- Regulate maximum driving hours
-- Weather-based speed limit adjustments</t>
+          <t>- Regular road maintenance
+- Stricter DUI checkpoints
+- Install rear-end collision warning systems
+- Install breathalyzer devices
+- Maintain current lighting standards</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Driver fatigue reduces reaction time and decision-making, interacting with lighting conditions and road geometry in systems theory to increase accident risk.</t>
+          <t>Drunk driving impairs human judgment and reaction time, interacting with vehicle control systems and road geometry to create hazardous situations in systems theory.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
@@ -755,27 +759,27 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Road Surface Treatment</t>
+          <t>Speed Checkpoint, Driver Safety Campaign</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>none</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>1155982.60</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>1155982.60</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
@@ -785,17 +789,17 @@
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>0.00 (Baseline 10.00, Intervention 10.00)</t>
+          <t>0.00 (Baseline 0.10, Intervention 0.10)</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
         <is>
-          <t>10.00</t>
+          <t>0.10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove ML predictor and update simulation workflow
Deleted ml_predictor.py and removed related dependencies from requirements.txt. Updated simulation.py to disable ML severity prediction and adjusted analysis.py for compatibility. Added generate_report_figures.py and generate_report_results.py for report generation and analysis. Updated accident_report.xlsx with new data.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -461,9 +461,9 @@
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="30" customWidth="1" min="22" max="22"/>
     <col width="30" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="30" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
     <col width="27" customWidth="1" min="27" max="27"/>
     <col width="30" customWidth="1" min="28" max="28"/>
     <col width="28" customWidth="1" min="29" max="29"/>
@@ -645,22 +645,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Vehicle-pedestrian collision</t>
+          <t>Head-on collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Bulhao, Labo, Camarines Norte</t>
+          <t>Malasugui, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1.74 seconds</t>
+          <t>3.35 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Reckless Driving</t>
+          <t>Fatigue</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -669,27 +669,31 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1206</v>
+        <v>1222</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>74.0</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Pedestrian</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>70</v>
-      </c>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Car 2</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1499</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>-55.4</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>wet</t>
+          <t>dry</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -699,29 +703,29 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Foggy</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>15</v>
+        <v>180</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>3.35</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>130842.55</t>
+          <t>1865020.57</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>severe</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>8.57</v>
+        <v>10</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -730,61 +734,61 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Maintain current lighting standards
-- Install anti-skid road surfaces
-- Increase traffic police presence
-- Install pedestrian crossings
-- Implement point-based license system</t>
+          <t>- Campaigns on driver fatigue awareness
+- Regular road maintenance
+- Improve lane markings
+- Regulate maximum driving hours
+- Maintain current lighting standards</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Reckless driving combines aggressive human behavior with vehicle capabilities and environmental factors in systems theory, leading to high-risk interactions.</t>
+          <t>Driver fatigue reduces reaction time and decision-making, interacting with lighting conditions and road geometry in systems theory to increase accident risk.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Road Surface Treatment</t>
+          <t>No interventions applied.</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>severe: 14, none: 4, moderate: 2</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>severe: 9, moderate: 6, none: 5</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>938230.12</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>720528.06</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
         <is>
-          <t>8.39</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>7.50</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add enhanced accident simulation report and figures
Added Enhanced_Paper.md detailing the development and validation of a road accident simulation and automatic reporting system for Labo, Camarines Norte. Updated accident_data.csv, accident_report.pdf, and accident_report.xlsx with new mechanical failure case data. Added report figures for severity comparison and impact force reduction to support quantitative analysis and intervention assessment.
</commit_message>
<xml_diff>
--- a/accident_report.xlsx
+++ b/accident_report.xlsx
@@ -441,7 +441,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -461,7 +461,7 @@
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="30" customWidth="1" min="22" max="22"/>
     <col width="30" customWidth="1" min="23" max="23"/>
-    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
     <col width="19" customWidth="1" min="25" max="25"/>
     <col width="23" customWidth="1" min="26" max="26"/>
     <col width="27" customWidth="1" min="27" max="27"/>
@@ -645,22 +645,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Head-on collision</t>
+          <t>Vehicle-pedestrian collision</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Malasugui, Labo, Camarines Norte</t>
+          <t>San Antonio, Labo, Camarines Norte</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>3.35 seconds</t>
+          <t>2.54 seconds</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Fatigue</t>
+          <t>Overspeeding</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -669,31 +669,27 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1222</v>
+        <v>1488</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Car 2</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>1499</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>-55.4</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Pedestrian</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>66</v>
+      </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>dry</t>
+          <t>wet</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -703,29 +699,29 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Rainy</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>180</v>
+        <v>15</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>3.35</t>
+          <t>2.54</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>1865020.57</t>
+          <t>117704.74</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>severe</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="T4" s="3" t="n">
-        <v>10</v>
+        <v>8.48</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
@@ -734,21 +730,21 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>- Campaigns on driver fatigue awareness
-- Regular road maintenance
-- Improve lane markings
-- Regulate maximum driving hours
-- Maintain current lighting standards</t>
+          <t>- Install anti-skid road surfaces
+- Increase speed limit enforcement
+- Maintain current lighting standards
+- Pedestrian safety education
+- Add speed bumps in high-risk areas</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Driver fatigue reduces reaction time and decision-making, interacting with lighting conditions and road geometry in systems theory to increase accident risk.</t>
+          <t>Overspeeding amplifies the impact of poor road conditions and reduces reaction time, leading to severe collisions in systems theory where human factors interact with vehicle dynamics and environmental constraints.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>No interventions applied.</t>
+          <t>Road Surface Treatment, Speed Checkpoint</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">

</xml_diff>